<commit_message>
Update example test file AdjustToContents
Update reference test file for example AdjustToContents.
After the style infrastructure switch, the styles part is saved differently.
No semantic change to the styles part.
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Examples/Misc/AdjustToContents.xlsx
+++ b/ClosedXML.Tests/Resource/Examples/Misc/AdjustToContents.xlsx
@@ -2949,161 +2949,121 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="0" formatCode=""/>
-  </x:numFmts>
-  <x:fonts count="3">
-    <x:font>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-    <x:font>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="30"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-    <x:font>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="20"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="2">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-  </x:fills>
-  <x:borders count="1">
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="none">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="none">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="none">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="none">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-  </x:borders>
-  <x:cellStyleXfs count="3">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellStyleXfs>
-  <x:cellXfs count="21">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="255" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="5" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="10" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="15" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="20" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="25" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="30" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="35" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="40" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="45" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="50" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="55" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="60" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="65" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="70" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="75" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="80" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="85" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellXfs>
-  <x:cellStyles count="1">
-    <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </x:cellStyles>
-</x:styleSheet>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="3">
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="30"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="20"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="22">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment textRotation="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment textRotation="10"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment textRotation="15"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment textRotation="20"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment textRotation="25"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment textRotation="30"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment textRotation="35"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment textRotation="40"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment textRotation="45"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment textRotation="50"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment textRotation="55"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment textRotation="60"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment textRotation="65"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment textRotation="70"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment textRotation="75"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment textRotation="80"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment textRotation="85"/>
+    </xf>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
+</styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3480,58 +3440,58 @@
       <x:c r="A1" s="3" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B1" s="0" t="s">
+      <x:c r="B1" s="4" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="C1" s="4" t="s">
+      <x:c r="C1" s="5" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="D1" s="5" t="s">
+      <x:c r="D1" s="6" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="E1" s="6" t="s">
+      <x:c r="E1" s="7" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="F1" s="7" t="s">
+      <x:c r="F1" s="8" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="G1" s="8" t="s">
+      <x:c r="G1" s="9" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="H1" s="9" t="s">
+      <x:c r="H1" s="10" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="I1" s="10" t="s">
+      <x:c r="I1" s="11" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="J1" s="11" t="s">
+      <x:c r="J1" s="12" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="K1" s="12" t="s">
+      <x:c r="K1" s="13" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="L1" s="13" t="s">
+      <x:c r="L1" s="14" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="M1" s="14" t="s">
+      <x:c r="M1" s="15" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="N1" s="15" t="s">
+      <x:c r="N1" s="16" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="O1" s="16" t="s">
+      <x:c r="O1" s="17" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="P1" s="17" t="s">
+      <x:c r="P1" s="18" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="Q1" s="18" t="s">
+      <x:c r="Q1" s="19" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="R1" s="19" t="s">
+      <x:c r="R1" s="20" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="S1" s="20" t="s">
+      <x:c r="S1" s="21" t="s">
         <x:v>24</x:v>
       </x:c>
     </x:row>
@@ -3577,58 +3537,58 @@
       <x:c r="A1" s="3" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B1" s="0" t="s">
+      <x:c r="B1" s="4" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="C1" s="4" t="s">
+      <x:c r="C1" s="5" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="D1" s="5" t="s">
+      <x:c r="D1" s="6" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="E1" s="6" t="s">
+      <x:c r="E1" s="7" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="F1" s="7" t="s">
+      <x:c r="F1" s="8" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="G1" s="8" t="s">
+      <x:c r="G1" s="9" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="H1" s="9" t="s">
+      <x:c r="H1" s="10" t="s">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="I1" s="10" t="s">
+      <x:c r="I1" s="11" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="J1" s="11" t="s">
+      <x:c r="J1" s="12" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="K1" s="12" t="s">
+      <x:c r="K1" s="13" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="L1" s="13" t="s">
+      <x:c r="L1" s="14" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="M1" s="14" t="s">
+      <x:c r="M1" s="15" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="N1" s="15" t="s">
+      <x:c r="N1" s="16" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="O1" s="16" t="s">
+      <x:c r="O1" s="17" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="P1" s="17" t="s">
+      <x:c r="P1" s="18" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="Q1" s="18" t="s">
+      <x:c r="Q1" s="19" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="R1" s="19" t="s">
+      <x:c r="R1" s="20" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="S1" s="20" t="s">
+      <x:c r="S1" s="21" t="s">
         <x:v>42</x:v>
       </x:c>
     </x:row>
@@ -3655,92 +3615,92 @@
       </x:c>
     </x:row>
     <x:row r="2" spans="1:1" ht="14.25" customHeight="1">
-      <x:c r="A2" s="0" t="s">
+      <x:c r="A2" s="4" t="s">
         <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:1" ht="21" customHeight="1">
-      <x:c r="A3" s="4" t="s">
+      <x:c r="A3" s="5" t="s">
         <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:1" ht="28.5" customHeight="1">
-      <x:c r="A4" s="5" t="s">
+      <x:c r="A4" s="6" t="s">
         <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:1" ht="34.5" customHeight="1">
-      <x:c r="A5" s="6" t="s">
+      <x:c r="A5" s="7" t="s">
         <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:1" ht="41.25" customHeight="1">
-      <x:c r="A6" s="7" t="s">
+      <x:c r="A6" s="8" t="s">
         <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:1" ht="47.25" customHeight="1">
-      <x:c r="A7" s="8" t="s">
+      <x:c r="A7" s="9" t="s">
         <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:1" ht="52.5" customHeight="1">
-      <x:c r="A8" s="9" t="s">
+      <x:c r="A8" s="10" t="s">
         <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:1" ht="57.75" customHeight="1">
-      <x:c r="A9" s="10" t="s">
+      <x:c r="A9" s="11" t="s">
         <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:1" ht="62.25" customHeight="1">
-      <x:c r="A10" s="11" t="s">
+      <x:c r="A10" s="12" t="s">
         <x:v>15</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:1" ht="66.75" customHeight="1">
-      <x:c r="A11" s="12" t="s">
+      <x:c r="A11" s="13" t="s">
         <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:1" ht="70.5" customHeight="1">
-      <x:c r="A12" s="13" t="s">
+      <x:c r="A12" s="14" t="s">
         <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:1" ht="73.5" customHeight="1">
-      <x:c r="A13" s="14" t="s">
+      <x:c r="A13" s="15" t="s">
         <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:1" ht="76.5" customHeight="1">
-      <x:c r="A14" s="15" t="s">
+      <x:c r="A14" s="16" t="s">
         <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:1" ht="78.75" customHeight="1">
-      <x:c r="A15" s="16" t="s">
+      <x:c r="A15" s="17" t="s">
         <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:1" ht="80.25" customHeight="1">
-      <x:c r="A16" s="17" t="s">
+      <x:c r="A16" s="18" t="s">
         <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:1" ht="81" customHeight="1">
-      <x:c r="A17" s="18" t="s">
+      <x:c r="A17" s="19" t="s">
         <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:1" ht="81" customHeight="1">
-      <x:c r="A18" s="19" t="s">
+      <x:c r="A18" s="20" t="s">
         <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:1" ht="81" customHeight="1">
-      <x:c r="A19" s="20" t="s">
+      <x:c r="A19" s="21" t="s">
         <x:v>24</x:v>
       </x:c>
     </x:row>
@@ -3767,92 +3727,92 @@
       </x:c>
     </x:row>
     <x:row r="2" spans="1:1" ht="59.25" customHeight="1">
-      <x:c r="A2" s="0" t="s">
+      <x:c r="A2" s="4" t="s">
         <x:v>43</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:1" ht="47.25" customHeight="1">
-      <x:c r="A3" s="4" t="s">
+      <x:c r="A3" s="5" t="s">
         <x:v>44</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:1" ht="75.75" customHeight="1">
-      <x:c r="A4" s="5" t="s">
+      <x:c r="A4" s="6" t="s">
         <x:v>45</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:1" ht="102.75" customHeight="1">
-      <x:c r="A5" s="6" t="s">
+      <x:c r="A5" s="7" t="s">
         <x:v>46</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:1" ht="129.75" customHeight="1">
-      <x:c r="A6" s="7" t="s">
+      <x:c r="A6" s="8" t="s">
         <x:v>47</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:1" ht="155.25" customHeight="1">
-      <x:c r="A7" s="8" t="s">
+      <x:c r="A7" s="9" t="s">
         <x:v>48</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:1" ht="180" customHeight="1">
-      <x:c r="A8" s="9" t="s">
+      <x:c r="A8" s="10" t="s">
         <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:1" ht="203.25" customHeight="1">
-      <x:c r="A9" s="10" t="s">
+      <x:c r="A9" s="11" t="s">
         <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:1" ht="225" customHeight="1">
-      <x:c r="A10" s="11" t="s">
+      <x:c r="A10" s="12" t="s">
         <x:v>51</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:1" ht="244.5" customHeight="1">
-      <x:c r="A11" s="12" t="s">
+      <x:c r="A11" s="13" t="s">
         <x:v>52</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:1" ht="263.25" customHeight="1">
-      <x:c r="A12" s="13" t="s">
+      <x:c r="A12" s="14" t="s">
         <x:v>53</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:1" ht="279" customHeight="1">
-      <x:c r="A13" s="14" t="s">
+      <x:c r="A13" s="15" t="s">
         <x:v>54</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:1" ht="293.25" customHeight="1">
-      <x:c r="A14" s="15" t="s">
+      <x:c r="A14" s="16" t="s">
         <x:v>55</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:1" ht="304.5" customHeight="1">
-      <x:c r="A15" s="16" t="s">
+      <x:c r="A15" s="17" t="s">
         <x:v>56</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:1" ht="314.25" customHeight="1">
-      <x:c r="A16" s="17" t="s">
+      <x:c r="A16" s="18" t="s">
         <x:v>57</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:1" ht="321" customHeight="1">
-      <x:c r="A17" s="18" t="s">
+      <x:c r="A17" s="19" t="s">
         <x:v>58</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:1" ht="325.5" customHeight="1">
-      <x:c r="A18" s="19" t="s">
+      <x:c r="A18" s="20" t="s">
         <x:v>59</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:1" ht="327.75" customHeight="1">
-      <x:c r="A19" s="20" t="s">
+      <x:c r="A19" s="21" t="s">
         <x:v>60</x:v>
       </x:c>
     </x:row>

</xml_diff>